<commit_message>
Daily scrape output - 2026-06-26
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_corners_current/pinnacle_corners_26062026.xlsx
+++ b/outputs/pinnacle_corners_current/pinnacle_corners_26062026.xlsx
@@ -472,7 +472,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>10.05</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="F2" t="n">
         <v>1.51</v>
@@ -498,10 +498,10 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>10.76</v>
+        <v>10.74</v>
       </c>
       <c r="F3" t="n">
-        <v>2.85</v>
+        <v>2.74</v>
       </c>
     </row>
     <row r="4">
@@ -680,7 +680,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>9.050000000000001</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="F10" t="n">
         <v>-1.66</v>
@@ -706,10 +706,10 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>9.289999999999999</v>
+        <v>9.32</v>
       </c>
       <c r="F11" t="n">
-        <v>3.04</v>
+        <v>3.42</v>
       </c>
     </row>
     <row r="12">
@@ -732,10 +732,10 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>8.81</v>
+        <v>8.67</v>
       </c>
       <c r="F12" t="n">
-        <v>0.18</v>
+        <v>-0.09</v>
       </c>
     </row>
     <row r="13">
@@ -888,10 +888,10 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>10.1</v>
+        <v>10.09</v>
       </c>
       <c r="F18" t="n">
-        <v>-4.4</v>
+        <v>-4.25</v>
       </c>
     </row>
     <row r="19">
@@ -914,10 +914,10 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>9.16</v>
+        <v>9.17</v>
       </c>
       <c r="F19" t="n">
-        <v>-2.14</v>
+        <v>-2.13</v>
       </c>
     </row>
     <row r="20">
@@ -940,10 +940,10 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>8.52</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="F20" t="n">
-        <v>-0.32</v>
+        <v>-0.18</v>
       </c>
     </row>
     <row r="21">
@@ -1021,7 +1021,7 @@
         <v>9.67</v>
       </c>
       <c r="F23" t="n">
-        <v>0.41</v>
+        <v>0.49</v>
       </c>
     </row>
     <row r="24">
@@ -1044,10 +1044,10 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>10.59</v>
+        <v>10.57</v>
       </c>
       <c r="F24" t="n">
-        <v>-0.67</v>
+        <v>-0.54</v>
       </c>
     </row>
     <row r="25">
@@ -1148,10 +1148,10 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>9.859999999999999</v>
+        <v>9.779999999999999</v>
       </c>
       <c r="F28" t="n">
-        <v>1.02</v>
+        <v>1.03</v>
       </c>
     </row>
     <row r="29">
@@ -1200,10 +1200,10 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>10.36</v>
+        <v>10.5</v>
       </c>
       <c r="F30" t="n">
-        <v>1.99</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="31">
@@ -1437,7 +1437,7 @@
         <v>10.83</v>
       </c>
       <c r="F39" t="n">
-        <v>-1.47</v>
+        <v>-1.46</v>
       </c>
     </row>
     <row r="40">
@@ -1512,10 +1512,10 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>11.16</v>
+        <v>11.13</v>
       </c>
       <c r="F42" t="n">
-        <v>2.03</v>
+        <v>2.01</v>
       </c>
     </row>
     <row r="43">
@@ -1538,10 +1538,10 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>10.95</v>
+        <v>10.83</v>
       </c>
       <c r="F43" t="n">
-        <v>0.05</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="44">
@@ -1668,10 +1668,10 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>10.5</v>
+        <v>10.49</v>
       </c>
       <c r="F48" t="n">
-        <v>1.66</v>
+        <v>1.67</v>
       </c>
     </row>
     <row r="49">
@@ -1720,10 +1720,10 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>10.51</v>
+        <v>10.07</v>
       </c>
       <c r="F50" t="n">
-        <v>1.69</v>
+        <v>1.71</v>
       </c>
     </row>
     <row r="51">
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>10.55</v>
+        <v>10.11</v>
       </c>
       <c r="F52" t="n">
-        <v>2.61</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="53">

</xml_diff>